<commit_message>
E4 (original model): rerun Set 1 (28 photos) and Set 2 (217 photos, detections only)
</commit_message>
<xml_diff>
--- a/experiments/E4_local_photos/RDD-Data/result/results.xlsx
+++ b/experiments/E4_local_photos/RDD-Data/result/results.xlsx
@@ -500,7 +500,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>28</t>
         </is>
       </c>
     </row>
@@ -548,7 +548,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>49</t>
         </is>
       </c>
     </row>
@@ -563,13 +563,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I21"/>
+  <dimension ref="A1:I29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
-    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
     <col width="37" customWidth="1" min="3" max="3"/>
-    <col width="20" customWidth="1" min="4" max="4"/>
+    <col width="30" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
     <col width="7" customWidth="1" min="7" max="7"/>
@@ -625,33 +625,33 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Saudi_0001.jpg</t>
+          <t>Saudi_000001.jpeg</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>partly (found 0, missed 1, false 2)</t>
+          <t>MISSED</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>D10 0.43, D00 0.27</t>
+          <t>nothing</t>
         </is>
       </c>
       <c r="E2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F2" t="n">
         <v>2</v>
       </c>
-      <c r="F2" t="n">
-        <v>1</v>
-      </c>
       <c r="G2" t="n">
         <v>0</v>
       </c>
       <c r="H2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I2" t="n">
         <v>2</v>
-      </c>
-      <c r="I2" t="n">
-        <v>1</v>
       </c>
     </row>
     <row r="3">
@@ -660,33 +660,33 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Saudi_0002.jpg</t>
+          <t>Saudi_0000010.jpeg</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>partly (found 0, missed 1, false 1)</t>
+          <t>MISSED</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>D20 0.49</t>
+          <t>nothing</t>
         </is>
       </c>
       <c r="E3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F3" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G3" t="n">
         <v>0</v>
       </c>
       <c r="H3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I3" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="4">
@@ -695,33 +695,33 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Saudi_0003.jpg</t>
+          <t>Saudi_0000011.jpeg</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>partly (found 1, missed 0, false 1)</t>
+          <t>partly (found 0, missed 1, false 3)</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>D10 0.64, D00 0.54</t>
+          <t>D00 0.56, D10 0.40, D00 0.27</t>
         </is>
       </c>
       <c r="E4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F4" t="n">
         <v>1</v>
       </c>
       <c r="G4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="I4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="5">
@@ -730,33 +730,33 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Saudi_0004.jpg</t>
+          <t>Saudi_0000012.jpeg</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>partly (found 1, missed 0, false 1)</t>
+          <t>MISSED</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>D20 0.80, D10 0.34</t>
+          <t>nothing</t>
         </is>
       </c>
       <c r="E5" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F5" t="n">
         <v>1</v>
       </c>
       <c r="G5" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H5" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="6">
@@ -765,33 +765,33 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Saudi_0005.jpg</t>
+          <t>Saudi_0000013.jpeg</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>partly (found 0, missed 1, false 1)</t>
+          <t>correct: no damage</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>D40 0.20</t>
+          <t>nothing</t>
         </is>
       </c>
       <c r="E6" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F6" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G6" t="n">
         <v>0</v>
       </c>
       <c r="H6" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I6" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="7">
@@ -800,33 +800,33 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Saudi_0006.jpg</t>
+          <t>Saudi_0000014.jpeg</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>partly (found 1, missed 0, false 1)</t>
+          <t>partly (found 0, missed 1, false 3)</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>D20 0.76, D40 0.15</t>
+          <t>D10 0.54, D10 0.31, D00 0.29</t>
         </is>
       </c>
       <c r="E7" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F7" t="n">
         <v>1</v>
       </c>
       <c r="G7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H7" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="I7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="8">
@@ -835,33 +835,33 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Saudi_0007.jpg</t>
+          <t>Saudi_0000015.jpeg</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>correct: no damage</t>
+          <t>partly (found 0, missed 3, false 1)</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>nothing</t>
+          <t>D10 0.38</t>
         </is>
       </c>
       <c r="E8" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F8" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="G8" t="n">
         <v>0</v>
       </c>
       <c r="H8" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I8" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="9">
@@ -870,33 +870,33 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Saudi_0008.jpg</t>
+          <t>Saudi_0000016.jpeg</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>partly (found 0, missed 1, false 2)</t>
+          <t>partly (found 0, missed 3, false 1)</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>D20 0.58, D10 0.32</t>
+          <t>D00 0.37</t>
         </is>
       </c>
       <c r="E9" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F9" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G9" t="n">
         <v>0</v>
       </c>
       <c r="H9" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I9" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="10">
@@ -905,33 +905,33 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Saudi_0009.jpg</t>
+          <t>Saudi_0000017.jpeg</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>partly (found 0, missed 1, false 1)</t>
+          <t>MISSED</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>D20 0.24</t>
+          <t>nothing</t>
         </is>
       </c>
       <c r="E10" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F10" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G10" t="n">
         <v>0</v>
       </c>
       <c r="H10" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I10" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="11">
@@ -940,33 +940,33 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Saudi_0010.jpg</t>
+          <t>Saudi_0000018.jpeg</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>all found</t>
+          <t>MISSED</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>D20 0.29</t>
+          <t>nothing</t>
         </is>
       </c>
       <c r="E11" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F11" t="n">
         <v>1</v>
       </c>
       <c r="G11" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H11" t="n">
         <v>0</v>
       </c>
       <c r="I11" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="12">
@@ -975,33 +975,33 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Saudi_0011.jpg</t>
+          <t>Saudi_0000019.jpeg</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>correct: no damage</t>
+          <t>partly (found 0, missed 1, false 1)</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>nothing</t>
+          <t>D40 0.16</t>
         </is>
       </c>
       <c r="E12" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F12" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G12" t="n">
         <v>0</v>
       </c>
       <c r="H12" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I12" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="13">
@@ -1010,33 +1010,33 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Saudi_0012.jpg</t>
+          <t>Saudi_000002.jpeg</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>FALSE ALARM</t>
+          <t>MISSED</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>D40 0.56</t>
+          <t>nothing</t>
         </is>
       </c>
       <c r="E13" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G13" t="n">
         <v>0</v>
       </c>
       <c r="H13" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="14">
@@ -1045,33 +1045,33 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Saudi_0013.jpg</t>
+          <t>Saudi_0000020.jpeg</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>correct: no damage</t>
+          <t>partly (found 0, missed 2, false 3)</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>nothing</t>
+          <t>D10 0.36, D00 0.31, D10 0.28</t>
         </is>
       </c>
       <c r="E14" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="F14" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G14" t="n">
         <v>0</v>
       </c>
       <c r="H14" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="I14" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="15">
@@ -1080,12 +1080,12 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Saudi_0014.jpg</t>
+          <t>Saudi_0000021.jpeg</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>correct: no damage</t>
+          <t>MISSED</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -1097,7 +1097,7 @@
         <v>0</v>
       </c>
       <c r="F15" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G15" t="n">
         <v>0</v>
@@ -1106,7 +1106,7 @@
         <v>0</v>
       </c>
       <c r="I15" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="16">
@@ -1115,33 +1115,33 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Saudi_0015.jpg</t>
+          <t>Saudi_0000022.jpeg</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>FALSE ALARM</t>
+          <t>MISSED</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>D40 0.61, D20 0.28</t>
+          <t>nothing</t>
         </is>
       </c>
       <c r="E16" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F16" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="G16" t="n">
         <v>0</v>
       </c>
       <c r="H16" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I16" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="17">
@@ -1150,33 +1150,33 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Saudi_0016.jpg</t>
+          <t>Saudi_0000023.jpeg</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>FALSE ALARM</t>
+          <t>MISSED</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>D20 0.27</t>
+          <t>nothing</t>
         </is>
       </c>
       <c r="E17" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F17" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G17" t="n">
         <v>0</v>
       </c>
       <c r="H17" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I17" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="18">
@@ -1185,24 +1185,24 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Saudi_0017.jpg</t>
+          <t>Saudi_0000024.jpeg</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>FALSE ALARM</t>
+          <t>partly (found 0, missed 2, false 1)</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>D00 0.60</t>
+          <t>D20 0.36</t>
         </is>
       </c>
       <c r="E18" t="n">
         <v>1</v>
       </c>
       <c r="F18" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G18" t="n">
         <v>0</v>
@@ -1211,7 +1211,7 @@
         <v>1</v>
       </c>
       <c r="I18" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="19">
@@ -1220,12 +1220,12 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Saudi_0018.jpg</t>
+          <t>Saudi_0000025.jpeg</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>correct: no damage</t>
+          <t>MISSED</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -1237,7 +1237,7 @@
         <v>0</v>
       </c>
       <c r="F19" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="G19" t="n">
         <v>0</v>
@@ -1246,7 +1246,7 @@
         <v>0</v>
       </c>
       <c r="I19" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="20">
@@ -1255,33 +1255,33 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Saudi_0019.jpg</t>
+          <t>Saudi_0000026.jpeg</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>FALSE ALARM</t>
+          <t>MISSED</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>D40 0.72</t>
+          <t>nothing</t>
         </is>
       </c>
       <c r="E20" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F20" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="G20" t="n">
         <v>0</v>
       </c>
       <c r="H20" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I20" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="21">
@@ -1290,33 +1290,313 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Saudi_0020.jpg</t>
+          <t>Saudi_0000027.jpeg</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>FALSE ALARM</t>
+          <t>all found</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>D00 0.44</t>
+          <t>D00 0.31</t>
         </is>
       </c>
       <c r="E21" t="n">
         <v>1</v>
       </c>
       <c r="F21" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G21" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H21" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I21" t="n">
         <v>0</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="1" t="n">
+        <v>20</v>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Saudi_0000028.jpeg</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>partly (found 0, missed 1, false 1)</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>D00 0.38</t>
+        </is>
+      </c>
+      <c r="E22" t="n">
+        <v>1</v>
+      </c>
+      <c r="F22" t="n">
+        <v>1</v>
+      </c>
+      <c r="G22" t="n">
+        <v>0</v>
+      </c>
+      <c r="H22" t="n">
+        <v>1</v>
+      </c>
+      <c r="I22" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="1" t="n">
+        <v>21</v>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Saudi_000003.jpeg</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>partly (found 0, missed 2, false 2)</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>D10 0.50, D10 0.41</t>
+        </is>
+      </c>
+      <c r="E23" t="n">
+        <v>2</v>
+      </c>
+      <c r="F23" t="n">
+        <v>2</v>
+      </c>
+      <c r="G23" t="n">
+        <v>0</v>
+      </c>
+      <c r="H23" t="n">
+        <v>2</v>
+      </c>
+      <c r="I23" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="1" t="n">
+        <v>22</v>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Saudi_000004.jpeg</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>partly (found 0, missed 1, false 1)</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>D00 0.34</t>
+        </is>
+      </c>
+      <c r="E24" t="n">
+        <v>1</v>
+      </c>
+      <c r="F24" t="n">
+        <v>1</v>
+      </c>
+      <c r="G24" t="n">
+        <v>0</v>
+      </c>
+      <c r="H24" t="n">
+        <v>1</v>
+      </c>
+      <c r="I24" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="1" t="n">
+        <v>23</v>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Saudi_000005.jpeg</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>partly (found 0, missed 1, false 1)</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>D00 0.28</t>
+        </is>
+      </c>
+      <c r="E25" t="n">
+        <v>1</v>
+      </c>
+      <c r="F25" t="n">
+        <v>1</v>
+      </c>
+      <c r="G25" t="n">
+        <v>0</v>
+      </c>
+      <c r="H25" t="n">
+        <v>1</v>
+      </c>
+      <c r="I25" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="1" t="n">
+        <v>24</v>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Saudi_000006.jpeg</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>MISSED</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>nothing</t>
+        </is>
+      </c>
+      <c r="E26" t="n">
+        <v>0</v>
+      </c>
+      <c r="F26" t="n">
+        <v>1</v>
+      </c>
+      <c r="G26" t="n">
+        <v>0</v>
+      </c>
+      <c r="H26" t="n">
+        <v>0</v>
+      </c>
+      <c r="I26" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="1" t="n">
+        <v>25</v>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Saudi_000007.jpeg</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>MISSED</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>nothing</t>
+        </is>
+      </c>
+      <c r="E27" t="n">
+        <v>0</v>
+      </c>
+      <c r="F27" t="n">
+        <v>1</v>
+      </c>
+      <c r="G27" t="n">
+        <v>0</v>
+      </c>
+      <c r="H27" t="n">
+        <v>0</v>
+      </c>
+      <c r="I27" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="1" t="n">
+        <v>26</v>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Saudi_000008.jpeg</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>MISSED</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>nothing</t>
+        </is>
+      </c>
+      <c r="E28" t="n">
+        <v>0</v>
+      </c>
+      <c r="F28" t="n">
+        <v>3</v>
+      </c>
+      <c r="G28" t="n">
+        <v>0</v>
+      </c>
+      <c r="H28" t="n">
+        <v>0</v>
+      </c>
+      <c r="I28" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="1" t="n">
+        <v>27</v>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Saudi_000009.jpeg</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>MISSED</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>nothing</t>
+        </is>
+      </c>
+      <c r="E29" t="n">
+        <v>0</v>
+      </c>
+      <c r="F29" t="n">
+        <v>2</v>
+      </c>
+      <c r="G29" t="n">
+        <v>0</v>
+      </c>
+      <c r="H29" t="n">
+        <v>0</v>
+      </c>
+      <c r="I29" t="n">
+        <v>2</v>
       </c>
     </row>
   </sheetData>
@@ -1335,14 +1615,14 @@
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
     <col width="11" customWidth="1" min="2" max="2"/>
-    <col width="11" customWidth="1" min="3" max="3"/>
-    <col width="21" customWidth="1" min="4" max="4"/>
-    <col width="21" customWidth="1" min="5" max="5"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="22" customWidth="1" min="5" max="5"/>
     <col width="5" customWidth="1" min="6" max="6"/>
     <col width="6" customWidth="1" min="7" max="7"/>
-    <col width="5" customWidth="1" min="8" max="8"/>
+    <col width="6" customWidth="1" min="8" max="8"/>
     <col width="12" customWidth="1" min="9" max="9"/>
-    <col width="21" customWidth="1" min="10" max="10"/>
+    <col width="22" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1402,28 +1682,28 @@
         <v>0.25</v>
       </c>
       <c r="C2" t="n">
-        <v>0.25</v>
+        <v>0.1111111111111111</v>
       </c>
       <c r="D2" t="n">
-        <v>0.3333333333333333</v>
+        <v>0.05555555555555555</v>
       </c>
       <c r="E2" t="n">
-        <v>0.2857142857142858</v>
+        <v>0.07407407407407407</v>
       </c>
       <c r="F2" t="n">
         <v>1</v>
       </c>
       <c r="G2" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="H2" t="n">
-        <v>2</v>
+        <v>17</v>
       </c>
       <c r="I2" t="n">
-        <v>3</v>
+        <v>18</v>
       </c>
       <c r="J2" t="n">
-        <v>0.425</v>
+        <v>0.0569334848649905</v>
       </c>
     </row>
     <row r="3">
@@ -1448,15 +1728,17 @@
         <v>0</v>
       </c>
       <c r="G3" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="H3" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="I3" t="n">
-        <v>0</v>
-      </c>
-      <c r="J3" t="inlineStr"/>
+        <v>8</v>
+      </c>
+      <c r="J3" t="n">
+        <v>0.02207155311994022</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="1" t="inlineStr">
@@ -1468,28 +1750,28 @@
         <v>0.24</v>
       </c>
       <c r="C4" t="n">
-        <v>0.375</v>
+        <v>0</v>
       </c>
       <c r="D4" t="n">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="E4" t="n">
-        <v>0.4285714285714285</v>
+        <v>0</v>
       </c>
       <c r="F4" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="G4" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="H4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I4" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="J4" t="n">
-        <v>0.5452117547355643</v>
+        <v>0.02671650055370985</v>
       </c>
     </row>
     <row r="5">
@@ -1514,15 +1796,17 @@
         <v>0</v>
       </c>
       <c r="G5" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="H5" t="n">
-        <v>0</v>
+        <v>21</v>
       </c>
       <c r="I5" t="n">
-        <v>0</v>
-      </c>
-      <c r="J5" t="inlineStr"/>
+        <v>21</v>
+      </c>
+      <c r="J5" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="1" t="inlineStr">
@@ -1532,28 +1816,28 @@
       </c>
       <c r="B6" t="inlineStr"/>
       <c r="C6" t="n">
-        <v>0.15625</v>
+        <v>0.02777777777777778</v>
       </c>
       <c r="D6" t="n">
-        <v>0.2083333333333333</v>
+        <v>0.01388888888888889</v>
       </c>
       <c r="E6" t="n">
-        <v>0.1785714285714286</v>
+        <v>0.01851851851851852</v>
       </c>
       <c r="F6" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="G6" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="H6" t="n">
-        <v>5</v>
+        <v>48</v>
       </c>
       <c r="I6" t="n">
-        <v>9</v>
+        <v>49</v>
       </c>
       <c r="J6" t="n">
-        <v>0.4851058773677821</v>
+        <v>0.02643038463466015</v>
       </c>
     </row>
   </sheetData>
@@ -1571,9 +1855,9 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
-    <col width="19" customWidth="1" min="2" max="2"/>
-    <col width="21" customWidth="1" min="3" max="3"/>
-    <col width="21" customWidth="1" min="4" max="4"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
     <col width="22" customWidth="1" min="5" max="5"/>
     <col width="29" customWidth="1" min="6" max="6"/>
     <col width="20" customWidth="1" min="7" max="7"/>
@@ -1636,31 +1920,31 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.25</v>
+        <v>0.1111111111111111</v>
       </c>
       <c r="C2" t="n">
-        <v>0.3333333333333333</v>
+        <v>0.05555555555555555</v>
       </c>
       <c r="D2" t="n">
-        <v>0.2857142857142858</v>
+        <v>0.07407407407407407</v>
       </c>
       <c r="E2" t="n">
         <v>0.6032482598607889</v>
       </c>
       <c r="F2" t="n">
-        <v>0.3532482598607889</v>
+        <v>0.4921371487496778</v>
       </c>
       <c r="G2" t="n">
         <v>0.4285714285714285</v>
       </c>
       <c r="H2" t="n">
-        <v>0.09523809523809518</v>
+        <v>0.3730158730158729</v>
       </c>
       <c r="I2" t="n">
         <v>0.5011243173787343</v>
       </c>
       <c r="J2" t="n">
-        <v>0.2154100316644486</v>
+        <v>0.4270502433046602</v>
       </c>
     </row>
     <row r="3">
@@ -1704,31 +1988,31 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.375</v>
+        <v>0</v>
       </c>
       <c r="C4" t="n">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="D4" t="n">
-        <v>0.4285714285714285</v>
+        <v>0</v>
       </c>
       <c r="E4" t="n">
         <v>0.6361940298507462</v>
       </c>
       <c r="F4" t="n">
-        <v>0.2611940298507462</v>
+        <v>0.6361940298507462</v>
       </c>
       <c r="G4" t="n">
         <v>0.5295031055900621</v>
       </c>
       <c r="H4" t="n">
-        <v>0.02950310559006208</v>
+        <v>0.5295031055900621</v>
       </c>
       <c r="I4" t="n">
         <v>0.5779661016949151</v>
       </c>
       <c r="J4" t="n">
-        <v>0.1493946731234866</v>
+        <v>0.5779661016949151</v>
       </c>
     </row>
     <row r="5">
@@ -1772,31 +2056,31 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.15625</v>
+        <v>0.02777777777777778</v>
       </c>
       <c r="C6" t="n">
-        <v>0.2083333333333333</v>
+        <v>0.01388888888888889</v>
       </c>
       <c r="D6" t="n">
-        <v>0.1785714285714286</v>
+        <v>0.01851851851851852</v>
       </c>
       <c r="E6" t="n">
         <v>0.5966236590911861</v>
       </c>
       <c r="F6" t="n">
-        <v>0.4403736590911861</v>
+        <v>0.5688458813134083</v>
       </c>
       <c r="G6" t="n">
         <v>0.5324479264696655</v>
       </c>
       <c r="H6" t="n">
-        <v>0.3241145931363322</v>
+        <v>0.5185590375807767</v>
       </c>
       <c r="I6" t="n">
         <v>0.5517365516374826</v>
       </c>
       <c r="J6" t="n">
-        <v>0.373165123066054</v>
+        <v>0.5332180331189641</v>
       </c>
     </row>
   </sheetData>
@@ -1831,7 +2115,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>20</v>
+        <v>28</v>
       </c>
     </row>
     <row r="3">
@@ -1841,7 +2125,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>15</v>
+        <v>12</v>
       </c>
     </row>
     <row r="4">
@@ -1851,7 +2135,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>5</v>
+        <v>16</v>
       </c>
     </row>
     <row r="5">
@@ -1861,7 +2145,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>9</v>
+        <v>27</v>
       </c>
     </row>
     <row r="6">
@@ -1871,7 +2155,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="7">
@@ -1881,7 +2165,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>11</v>
+        <v>1</v>
       </c>
     </row>
     <row r="8">
@@ -1891,7 +2175,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -1926,7 +2210,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
     </row>
     <row r="3">
@@ -1936,7 +2220,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
     </row>
     <row r="4">
@@ -1946,7 +2230,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
     </row>
     <row r="5">
@@ -1956,7 +2240,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>